<commit_message>
Phase 4: cash flow statement and supporting schedules
</commit_message>
<xml_diff>
--- a/model/3 statement model .xlsx
+++ b/model/3 statement model .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ravishagosain/Desktop/WorkX/Finance/projects/3 statement model/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D92D3D-4957-7040-B9EC-C5F991EA7283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F114AF10-D75F-2E42-A8D8-2EF5703215AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{C2ABDD43-7712-494D-BFB8-6BE793A7A1EB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="11" xr2:uid="{C2ABDD43-7712-494D-BFB8-6BE793A7A1EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,13 @@
     <sheet name="IS" sheetId="3" r:id="rId3"/>
     <sheet name="BS" sheetId="4" r:id="rId4"/>
     <sheet name="CFS" sheetId="5" r:id="rId5"/>
-    <sheet name="Check" sheetId="6" r:id="rId6"/>
-    <sheet name="PP&amp;E Sch" sheetId="7" r:id="rId7"/>
-    <sheet name="WC Sch" sheetId="8" r:id="rId8"/>
-    <sheet name="Sheet1" sheetId="12" r:id="rId9"/>
-    <sheet name="WACC" sheetId="9" r:id="rId10"/>
-    <sheet name="DCF" sheetId="10" r:id="rId11"/>
-    <sheet name="Sensitivity" sheetId="11" r:id="rId12"/>
+    <sheet name="PP&amp;E Sch" sheetId="7" r:id="rId6"/>
+    <sheet name="WC Sch" sheetId="8" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="12" r:id="rId8"/>
+    <sheet name="WACC" sheetId="9" r:id="rId9"/>
+    <sheet name="DCF" sheetId="10" r:id="rId10"/>
+    <sheet name="Sensitivity" sheetId="11" r:id="rId11"/>
+    <sheet name="Check" sheetId="6" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="193">
   <si>
     <t>Infosys Limited</t>
   </si>
@@ -582,9 +582,6 @@
     <t>PP&amp;E Schedule (₹ Crores)</t>
   </si>
   <si>
-    <t>Gross PP&amp;E</t>
-  </si>
-  <si>
     <t>Closing gross PP&amp;E</t>
   </si>
   <si>
@@ -625,6 +622,9 @@
   </si>
   <si>
     <t>Provisions % of Revenue</t>
+  </si>
+  <si>
+    <t>WC Schedule (₹ Crores)</t>
   </si>
 </sst>
 </file>
@@ -745,7 +745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -798,12 +798,15 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1155,15 +1158,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD350CFE-D0BB-9A48-980A-212CF0B3318D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89457251-7A5A-794C-96B2-478D35C4F3B9}">
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
@@ -1175,7 +1169,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC98C098-C6A3-5B4B-9CE0-7F4E98F70504}">
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
@@ -1188,6 +1182,96 @@
     <col min="38" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90E68197-B81D-A946-87FA-197633624652}">
+  <sheetPr>
+    <tabColor theme="2" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A2:J3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="str">
+        <f>BS!F4</f>
+        <v>FY26E</v>
+      </c>
+      <c r="G2" s="3" t="str">
+        <f>BS!G4</f>
+        <v xml:space="preserve">FY27E </v>
+      </c>
+      <c r="H2" s="3" t="str">
+        <f>BS!H4</f>
+        <v>FY28E</v>
+      </c>
+      <c r="I2" s="3" t="str">
+        <f>BS!I4</f>
+        <v>FY29E</v>
+      </c>
+      <c r="J2" s="3" t="str">
+        <f>BS!J4</f>
+        <v>FY30E</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C3" s="30">
+        <f>BS!C33-BS!C63</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="30">
+        <f>BS!D33-BS!D63</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="30">
+        <f>BS!E33-BS!E63</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="30">
+        <f>BS!F33-BS!F63</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="30">
+        <f>BS!G33-BS!G63</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="30">
+        <f>BS!H33-BS!H63</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="30">
+        <f>BS!I33-BS!I63</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="30">
+        <f>BS!J33-BS!J63</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C3:J3">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1567,7 +1651,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C20" s="19">
         <v>8.5000000000000006E-2</v>
@@ -1599,7 +1683,7 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C22" s="19">
         <v>0.65</v>
@@ -1630,8 +1714,8 @@
       <c r="E23" s="16"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="35" t="s">
-        <v>191</v>
+      <c r="A24" t="s">
+        <v>190</v>
       </c>
       <c r="C24" s="19">
         <v>0.3</v>
@@ -1662,8 +1746,8 @@
       <c r="E25" s="16"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="35" t="s">
-        <v>192</v>
+      <c r="A26" t="s">
+        <v>191</v>
       </c>
       <c r="C26" s="19">
         <v>0.01</v>
@@ -2096,23 +2180,23 @@
       <c r="E16" s="6">
         <v>4812</v>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="30">
         <f>F5*(E16/E5)</f>
         <v>5148.8400000000011</v>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="30">
         <f t="shared" ref="G16:J16" si="8">G5*(F16/F5)</f>
         <v>5509.2588000000014</v>
       </c>
-      <c r="H16" s="32">
+      <c r="H16" s="30">
         <f t="shared" si="8"/>
         <v>5883.8883984000013</v>
       </c>
-      <c r="I16" s="32">
+      <c r="I16" s="30">
         <f t="shared" si="8"/>
         <v>6266.3411442960014</v>
       </c>
-      <c r="J16" s="32">
+      <c r="J16" s="30">
         <f t="shared" si="8"/>
         <v>6673.6533186752413</v>
       </c>
@@ -2806,48 +2890,48 @@
       </c>
       <c r="C8" s="31">
         <f>'PP&amp;E Sch'!C14</f>
-        <v>11656</v>
+        <v>13346</v>
       </c>
       <c r="D8" s="31">
         <f>'PP&amp;E Sch'!D14</f>
-        <v>10813</v>
+        <v>12370</v>
       </c>
       <c r="E8" s="31">
         <f>'PP&amp;E Sch'!E14</f>
-        <v>10070</v>
+        <v>11778</v>
       </c>
       <c r="F8" s="31">
         <f>'PP&amp;E Sch'!F14</f>
-        <v>10163.125199999999</v>
+        <v>11559.940199999997</v>
       </c>
       <c r="G8" s="31">
         <f>'PP&amp;E Sch'!G14</f>
-        <v>10219.626546999996</v>
+        <v>11305.256547000001</v>
       </c>
       <c r="H8" s="31">
         <f>'PP&amp;E Sch'!H14</f>
-        <v>10331.363640295996</v>
+        <v>11105.808640296003</v>
       </c>
       <c r="I8" s="31">
         <f>'PP&amp;E Sch'!I14</f>
-        <v>10427.754899698761</v>
+        <v>10891.01489969877</v>
       </c>
       <c r="J8" s="31">
         <f>'PP&amp;E Sch'!J14</f>
-        <v>10529.558554997053</v>
+        <v>10681.633554997061</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="33">
+      <c r="C9" s="32">
         <v>3561</v>
       </c>
-      <c r="D9" s="33">
+      <c r="D9" s="32">
         <v>6552</v>
       </c>
-      <c r="E9" s="33">
+      <c r="E9" s="32">
         <v>6311</v>
       </c>
       <c r="F9" s="30">
@@ -2875,13 +2959,13 @@
       <c r="A10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="33">
+      <c r="C10" s="32">
         <v>275</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="32">
         <v>293</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="32">
         <v>814</v>
       </c>
       <c r="F10" s="30">
@@ -2909,13 +2993,13 @@
       <c r="A11" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="33">
+      <c r="C11" s="32">
         <v>211</v>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="32">
         <v>7303</v>
       </c>
-      <c r="E11" s="33">
+      <c r="E11" s="32">
         <v>10106</v>
       </c>
       <c r="F11" s="30">
@@ -2943,13 +3027,13 @@
       <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="33">
+      <c r="C12" s="32">
         <v>3</v>
       </c>
-      <c r="D12" s="33">
+      <c r="D12" s="32">
         <v>1397</v>
       </c>
-      <c r="E12" s="33">
+      <c r="E12" s="32">
         <v>2766</v>
       </c>
       <c r="F12" s="30">
@@ -2977,9 +3061,9 @@
       <c r="A13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
       <c r="F13" s="30"/>
       <c r="G13" s="30"/>
       <c r="H13" s="30"/>
@@ -2990,13 +3074,13 @@
       <c r="A14" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="33">
+      <c r="C14" s="32">
         <v>23686</v>
       </c>
-      <c r="D14" s="33">
+      <c r="D14" s="32">
         <v>11708</v>
       </c>
-      <c r="E14" s="33">
+      <c r="E14" s="32">
         <v>11059</v>
       </c>
       <c r="F14" s="30">
@@ -3024,13 +3108,13 @@
       <c r="A15" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="32">
         <v>39</v>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="32">
         <v>34</v>
       </c>
-      <c r="E15" s="33">
+      <c r="E15" s="32">
         <v>16</v>
       </c>
       <c r="F15" s="30">
@@ -3058,13 +3142,13 @@
       <c r="A16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="33">
+      <c r="C16" s="32">
         <v>1341</v>
       </c>
-      <c r="D16" s="33">
+      <c r="D16" s="32">
         <v>3105</v>
       </c>
-      <c r="E16" s="33">
+      <c r="E16" s="32">
         <v>3511</v>
       </c>
       <c r="F16" s="30">
@@ -3092,13 +3176,13 @@
       <c r="A17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="33">
+      <c r="C17" s="32">
         <v>779</v>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="32">
         <v>454</v>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="32">
         <v>1108</v>
       </c>
       <c r="F17" s="30">
@@ -3126,13 +3210,13 @@
       <c r="A18" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="32">
         <v>5916</v>
       </c>
-      <c r="D18" s="33">
+      <c r="D18" s="32">
         <v>3045</v>
       </c>
-      <c r="E18" s="33">
+      <c r="E18" s="32">
         <v>1622</v>
       </c>
       <c r="F18" s="30">
@@ -3160,32 +3244,32 @@
       <c r="A19" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="33">
+      <c r="C19" s="32">
         <v>1788</v>
       </c>
-      <c r="D19" s="33">
+      <c r="D19" s="32">
         <v>2121</v>
       </c>
-      <c r="E19" s="33">
+      <c r="E19" s="32">
         <v>2713</v>
       </c>
-      <c r="F19" s="30">
+      <c r="F19" s="38">
+        <f>E19</f>
+        <v>2713</v>
+      </c>
+      <c r="G19" s="38">
         <f t="shared" si="5"/>
         <v>2713</v>
       </c>
-      <c r="G19" s="30">
+      <c r="H19" s="38">
         <f t="shared" si="5"/>
         <v>2713</v>
       </c>
-      <c r="H19" s="30">
+      <c r="I19" s="38">
         <f t="shared" si="5"/>
         <v>2713</v>
       </c>
-      <c r="I19" s="30">
-        <f t="shared" si="5"/>
-        <v>2713</v>
-      </c>
-      <c r="J19" s="30">
+      <c r="J19" s="38">
         <f t="shared" si="5"/>
         <v>2713</v>
       </c>
@@ -3195,39 +3279,42 @@
         <v>38</v>
       </c>
       <c r="C20" s="34">
-        <v>49255</v>
+        <f t="shared" ref="C20:E20" si="6">SUM(C8:C19)</f>
+        <v>50945</v>
       </c>
       <c r="D20" s="34">
+        <f t="shared" si="6"/>
         <v>48382</v>
       </c>
       <c r="E20" s="34">
+        <f t="shared" si="6"/>
         <v>51804</v>
       </c>
-      <c r="F20" s="36">
+      <c r="F20" s="34">
         <f>SUM(F8:F19)</f>
-        <v>50107.60226</v>
-      </c>
-      <c r="G20" s="36">
-        <f t="shared" si="5"/>
-        <v>50107.60226</v>
-      </c>
-      <c r="H20" s="36">
-        <f t="shared" si="5"/>
-        <v>50107.60226</v>
-      </c>
-      <c r="I20" s="36">
-        <f t="shared" si="5"/>
-        <v>50107.60226</v>
-      </c>
-      <c r="J20" s="36">
-        <f t="shared" si="5"/>
-        <v>50107.60226</v>
+        <v>51504.417260000002</v>
+      </c>
+      <c r="G20" s="34">
+        <f t="shared" ref="G20:J20" si="7">SUM(G8:G19)</f>
+        <v>51301.0070012</v>
+      </c>
+      <c r="H20" s="34">
+        <f t="shared" si="7"/>
+        <v>51184.748606991809</v>
+      </c>
+      <c r="I20" s="34">
+        <f t="shared" si="7"/>
+        <v>51039.041013395741</v>
+      </c>
+      <c r="J20" s="34">
+        <f t="shared" si="7"/>
+        <v>50910.845607126932</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
       <c r="F21" s="30"/>
       <c r="G21" s="30"/>
       <c r="H21" s="30"/>
@@ -3238,9 +3325,9 @@
       <c r="A22" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
       <c r="F22" s="30"/>
       <c r="G22" s="30"/>
       <c r="H22" s="30"/>
@@ -3251,9 +3338,9 @@
       <c r="A23" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="33"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="33"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
       <c r="F23" s="30"/>
       <c r="G23" s="30"/>
       <c r="H23" s="30"/>
@@ -3264,13 +3351,13 @@
       <c r="A24" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="33">
+      <c r="C24" s="32">
         <v>4476</v>
       </c>
-      <c r="D24" s="33">
+      <c r="D24" s="32">
         <v>12915</v>
       </c>
-      <c r="E24" s="33">
+      <c r="E24" s="32">
         <v>12482</v>
       </c>
       <c r="F24" s="30">
@@ -3278,19 +3365,19 @@
         <v>12482</v>
       </c>
       <c r="G24" s="30">
-        <f t="shared" ref="G24:J24" si="6">F24</f>
+        <f t="shared" ref="G24:J24" si="8">F24</f>
         <v>12482</v>
       </c>
       <c r="H24" s="30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>12482</v>
       </c>
       <c r="I24" s="30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>12482</v>
       </c>
       <c r="J24" s="30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>12482</v>
       </c>
     </row>
@@ -3298,13 +3385,13 @@
       <c r="A25" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="33">
+      <c r="C25" s="32">
         <v>20773</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="32">
         <v>30193</v>
       </c>
-      <c r="E25" s="33">
+      <c r="E25" s="32">
         <v>31158</v>
       </c>
       <c r="F25" s="31">
@@ -3332,32 +3419,50 @@
       <c r="A26" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="33">
+      <c r="C26" s="31">
+        <f>CFS!C79</f>
         <v>6534</v>
       </c>
-      <c r="D26" s="33">
+      <c r="D26" s="31">
+        <f>CFS!D79</f>
         <v>14786</v>
       </c>
-      <c r="E26" s="33">
+      <c r="E26" s="31">
+        <f>CFS!E79</f>
         <v>24455</v>
       </c>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="30"/>
+      <c r="F26" s="31">
+        <f>CFS!F79</f>
+        <v>34335.04869016986</v>
+      </c>
+      <c r="G26" s="31">
+        <f>CFS!G79</f>
+        <v>45207.613983999516</v>
+      </c>
+      <c r="H26" s="31">
+        <f>CFS!H79</f>
+        <v>55879.739328854928</v>
+      </c>
+      <c r="I26" s="31">
+        <f>CFS!I79</f>
+        <v>68366.711390721961</v>
+      </c>
+      <c r="J26" s="31">
+        <f>CFS!J79</f>
+        <v>81056.844361363954</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="33">
+      <c r="C27" s="32">
         <v>291</v>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="32">
         <v>248</v>
       </c>
-      <c r="E27" s="33">
+      <c r="E27" s="32">
         <v>249</v>
       </c>
       <c r="F27" s="30">
@@ -3365,19 +3470,19 @@
         <v>249</v>
       </c>
       <c r="G27" s="30">
-        <f t="shared" ref="G27:J27" si="7">F27</f>
+        <f t="shared" ref="G27:J27" si="9">F27</f>
         <v>249</v>
       </c>
       <c r="H27" s="30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>249</v>
       </c>
       <c r="I27" s="30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>249</v>
       </c>
       <c r="J27" s="30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>249</v>
       </c>
     </row>
@@ -3385,33 +3490,33 @@
       <c r="A28" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="33">
+      <c r="C28" s="32">
         <v>9088</v>
       </c>
-      <c r="D28" s="33">
+      <c r="D28" s="32">
         <v>12085</v>
       </c>
-      <c r="E28" s="33">
+      <c r="E28" s="32">
         <v>13840</v>
       </c>
       <c r="F28" s="30">
-        <f t="shared" ref="F28:J31" si="8">E28</f>
+        <f t="shared" ref="F28:J31" si="10">E28</f>
         <v>13840</v>
       </c>
       <c r="G28" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>13840</v>
       </c>
       <c r="H28" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>13840</v>
       </c>
       <c r="I28" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>13840</v>
       </c>
       <c r="J28" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>13840</v>
       </c>
     </row>
@@ -3419,34 +3524,34 @@
       <c r="A29" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C29" s="33">
+      <c r="C29" s="32">
         <f>-C30</f>
         <v>-10920</v>
       </c>
-      <c r="D29" s="33">
+      <c r="D29" s="32">
         <v>6397</v>
       </c>
-      <c r="E29" s="33">
+      <c r="E29" s="32">
         <v>2975</v>
       </c>
       <c r="F29" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>2975</v>
       </c>
       <c r="G29" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>2975</v>
       </c>
       <c r="H29" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>2975</v>
       </c>
       <c r="I29" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>2975</v>
       </c>
       <c r="J29" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>2975</v>
       </c>
     </row>
@@ -3454,33 +3559,33 @@
       <c r="A30" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C30" s="32">
         <v>10920</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="32">
         <v>12808</v>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="32">
         <v>11940</v>
       </c>
       <c r="F30" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11940</v>
       </c>
       <c r="G30" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11940</v>
       </c>
       <c r="H30" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11940</v>
       </c>
       <c r="I30" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11940</v>
       </c>
       <c r="J30" s="30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11940</v>
       </c>
     </row>
@@ -3488,40 +3593,40 @@
       <c r="A31" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="34">
+      <c r="C31" s="33">
         <v>52082</v>
       </c>
-      <c r="D31" s="34">
+      <c r="D31" s="33">
         <v>89432</v>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="33">
         <v>97099</v>
       </c>
-      <c r="F31" s="36">
+      <c r="F31" s="34">
         <f>SUM(F24:F30)</f>
-        <v>74932.441095890419</v>
-      </c>
-      <c r="G31" s="36">
-        <f t="shared" si="8"/>
-        <v>74932.441095890419</v>
-      </c>
-      <c r="H31" s="36">
-        <f t="shared" si="8"/>
-        <v>74932.441095890419</v>
-      </c>
-      <c r="I31" s="36">
-        <f t="shared" si="8"/>
-        <v>74932.441095890419</v>
-      </c>
-      <c r="J31" s="36">
-        <f t="shared" si="8"/>
-        <v>74932.441095890419</v>
+        <v>109267.48978606027</v>
+      </c>
+      <c r="G31" s="34">
+        <f t="shared" ref="G31:J31" si="11">SUM(G24:G30)</f>
+        <v>121970.05321413651</v>
+      </c>
+      <c r="H31" s="34">
+        <f t="shared" si="11"/>
+        <v>135040.97642664122</v>
+      </c>
+      <c r="I31" s="34">
+        <f t="shared" si="11"/>
+        <v>149395.32980552898</v>
+      </c>
+      <c r="J31" s="34">
+        <f t="shared" si="11"/>
+        <v>164655.73297313342</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C32" s="33"/>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
       <c r="F32" s="30"/>
       <c r="G32" s="30"/>
       <c r="H32" s="30"/>
@@ -3532,25 +3637,40 @@
       <c r="A33" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C33" s="34">
+      <c r="C33" s="33">
         <v>101337</v>
       </c>
-      <c r="D33" s="34">
+      <c r="D33" s="33">
         <v>137814</v>
       </c>
-      <c r="E33" s="34">
+      <c r="E33" s="33">
         <v>148903</v>
       </c>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
+      <c r="F33" s="34">
+        <f>SUM(F20,F31)</f>
+        <v>160771.90704606025</v>
+      </c>
+      <c r="G33" s="34">
+        <f t="shared" ref="G33:J33" si="12">SUM(G20,G31)</f>
+        <v>173271.0602153365</v>
+      </c>
+      <c r="H33" s="34">
+        <f t="shared" si="12"/>
+        <v>186225.72503363303</v>
+      </c>
+      <c r="I33" s="34">
+        <f t="shared" si="12"/>
+        <v>200434.37081892471</v>
+      </c>
+      <c r="J33" s="34">
+        <f t="shared" si="12"/>
+        <v>215566.57858026034</v>
+      </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
       <c r="F34" s="30"/>
       <c r="G34" s="30"/>
       <c r="H34" s="30"/>
@@ -3561,9 +3681,9 @@
       <c r="A35" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
       <c r="F35" s="30"/>
       <c r="G35" s="30"/>
       <c r="H35" s="30"/>
@@ -3571,9 +3691,9 @@
       <c r="J35" s="30"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
       <c r="F36" s="30"/>
       <c r="G36" s="30"/>
       <c r="H36" s="30"/>
@@ -3584,13 +3704,13 @@
       <c r="A37" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="33">
+      <c r="C37" s="32">
         <v>2074</v>
       </c>
-      <c r="D37" s="33">
+      <c r="D37" s="32">
         <v>2071</v>
       </c>
-      <c r="E37" s="33">
+      <c r="E37" s="32">
         <v>2073</v>
       </c>
       <c r="F37" s="30">
@@ -3598,19 +3718,19 @@
         <v>2073</v>
       </c>
       <c r="G37" s="30">
-        <f t="shared" ref="G37:J37" si="9">F37</f>
+        <f t="shared" ref="G37:J37" si="13">F37</f>
         <v>2073</v>
       </c>
       <c r="H37" s="30">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>2073</v>
       </c>
       <c r="I37" s="30">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>2073</v>
       </c>
       <c r="J37" s="30">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>2073</v>
       </c>
     </row>
@@ -3618,13 +3738,13 @@
       <c r="A38" t="s">
         <v>47</v>
       </c>
-      <c r="C38" s="33">
+      <c r="C38" s="32">
         <v>65671</v>
       </c>
-      <c r="D38" s="33">
+      <c r="D38" s="32">
         <v>86045</v>
       </c>
-      <c r="E38" s="33">
+      <c r="E38" s="32">
         <v>93745</v>
       </c>
       <c r="F38" s="30">
@@ -3632,75 +3752,75 @@
         <v>104971.5746488</v>
       </c>
       <c r="G38" s="30">
-        <f>F38+IS!G27-(IS!G27*Assumptions!G21)</f>
-        <v>139427.17436728001</v>
+        <f>F38+IS!G27-(IS!G27*Assumptions!G22)</f>
+        <v>117031.034550268</v>
       </c>
       <c r="H38" s="30">
-        <f>G38+IS!H27-(IS!H27*Assumptions!H21)</f>
-        <v>176369.24837834563</v>
+        <f>G38+IS!H27-(IS!H27*Assumptions!H22)</f>
+        <v>129960.76045414098</v>
       </c>
       <c r="I38" s="30">
-        <f>H38+IS!I27-(IS!I27*Assumptions!I21)</f>
-        <v>215712.55720013048</v>
+        <f>H38+IS!I27-(IS!I27*Assumptions!I22)</f>
+        <v>143730.91854176568</v>
       </c>
       <c r="J38" s="30">
-        <f>I38+IS!J27-(IS!J27*Assumptions!J21)</f>
-        <v>257613.18109533135</v>
+        <f>I38+IS!J27-(IS!J27*Assumptions!J22)</f>
+        <v>158396.13690508599</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33">
-        <f t="shared" ref="D39:J39" si="10">E37+E38</f>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32">
+        <f t="shared" ref="E39:J39" si="14">E37+E38</f>
         <v>95818</v>
       </c>
-      <c r="F39" s="33">
-        <f t="shared" si="10"/>
+      <c r="F39" s="32">
+        <f>F37+F38</f>
         <v>107044.5746488</v>
       </c>
-      <c r="G39" s="33">
-        <f t="shared" si="10"/>
-        <v>141500.17436728001</v>
-      </c>
-      <c r="H39" s="33">
-        <f t="shared" si="10"/>
-        <v>178442.24837834563</v>
-      </c>
-      <c r="I39" s="33">
-        <f t="shared" si="10"/>
-        <v>217785.55720013048</v>
-      </c>
-      <c r="J39" s="33">
-        <f t="shared" si="10"/>
-        <v>259686.18109533135</v>
+      <c r="G39" s="32">
+        <f t="shared" si="14"/>
+        <v>119104.034550268</v>
+      </c>
+      <c r="H39" s="32">
+        <f t="shared" si="14"/>
+        <v>132033.76045414098</v>
+      </c>
+      <c r="I39" s="32">
+        <f t="shared" si="14"/>
+        <v>145803.91854176568</v>
+      </c>
+      <c r="J39" s="32">
+        <f t="shared" si="14"/>
+        <v>160469.13690508599</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>65</v>
       </c>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33">
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32">
         <v>385</v>
       </c>
-      <c r="F40" s="33">
+      <c r="F40" s="32">
         <v>385</v>
       </c>
-      <c r="G40" s="33">
+      <c r="G40" s="32">
         <v>385</v>
       </c>
-      <c r="H40" s="33">
+      <c r="H40" s="32">
         <v>385</v>
       </c>
-      <c r="I40" s="33">
+      <c r="I40" s="32">
         <v>385</v>
       </c>
-      <c r="J40" s="33">
+      <c r="J40" s="32">
         <v>385</v>
       </c>
     </row>
@@ -3708,40 +3828,41 @@
       <c r="A41" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C41" s="34">
+      <c r="C41" s="33">
         <v>67745</v>
       </c>
-      <c r="D41" s="34">
+      <c r="D41" s="33">
         <v>88461</v>
       </c>
-      <c r="E41" s="34">
+      <c r="E41" s="33">
+        <f>SUM(E39:E40)</f>
         <v>96203</v>
       </c>
-      <c r="F41" s="30">
+      <c r="F41" s="34">
         <f>SUM(F39:F40)</f>
         <v>107429.5746488</v>
       </c>
-      <c r="G41" s="30">
-        <f t="shared" ref="G41:J41" si="11">SUM(G39:G40)</f>
-        <v>141885.17436728001</v>
-      </c>
-      <c r="H41" s="30">
-        <f t="shared" si="11"/>
-        <v>178827.24837834563</v>
-      </c>
-      <c r="I41" s="30">
-        <f t="shared" si="11"/>
-        <v>218170.55720013048</v>
-      </c>
-      <c r="J41" s="30">
-        <f t="shared" si="11"/>
-        <v>260071.18109533135</v>
+      <c r="G41" s="34">
+        <f t="shared" ref="G41:J41" si="15">SUM(G39:G40)</f>
+        <v>119489.034550268</v>
+      </c>
+      <c r="H41" s="34">
+        <f t="shared" si="15"/>
+        <v>132418.76045414098</v>
+      </c>
+      <c r="I41" s="34">
+        <f t="shared" si="15"/>
+        <v>146188.91854176568</v>
+      </c>
+      <c r="J41" s="34">
+        <f t="shared" si="15"/>
+        <v>160854.13690508599</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C42" s="33"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="33"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
       <c r="F42" s="30"/>
       <c r="G42" s="30"/>
       <c r="H42" s="30"/>
@@ -3752,9 +3873,9 @@
       <c r="A43" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C43" s="33"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="33"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
       <c r="F43" s="30"/>
       <c r="G43" s="30"/>
       <c r="H43" s="30"/>
@@ -3762,9 +3883,9 @@
       <c r="J43" s="30"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C44" s="33"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="33"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
       <c r="F44" s="30"/>
       <c r="G44" s="30"/>
       <c r="H44" s="30"/>
@@ -3775,9 +3896,9 @@
       <c r="A45" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="33"/>
-      <c r="D45" s="33"/>
-      <c r="E45" s="33"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
       <c r="F45" s="30"/>
       <c r="G45" s="30"/>
       <c r="H45" s="30"/>
@@ -3788,9 +3909,9 @@
       <c r="A46" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C46" s="33"/>
-      <c r="D46" s="33"/>
-      <c r="E46" s="33"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="32"/>
+      <c r="E46" s="32"/>
       <c r="F46" s="30"/>
       <c r="G46" s="30"/>
       <c r="H46" s="30"/>
@@ -3801,28 +3922,28 @@
       <c r="A47" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C47" s="33">
+      <c r="C47" s="32">
         <v>3553</v>
       </c>
-      <c r="D47" s="33">
+      <c r="D47" s="32">
         <v>6400</v>
       </c>
-      <c r="E47" s="33">
+      <c r="E47" s="32">
         <v>5772</v>
       </c>
-      <c r="F47" s="32">
+      <c r="F47" s="30">
         <v>5772</v>
       </c>
-      <c r="G47" s="32">
+      <c r="G47" s="30">
         <v>5772</v>
       </c>
-      <c r="H47" s="32">
+      <c r="H47" s="30">
         <v>5772</v>
       </c>
-      <c r="I47" s="32">
+      <c r="I47" s="30">
         <v>5772</v>
       </c>
-      <c r="J47" s="32">
+      <c r="J47" s="30">
         <v>5772</v>
       </c>
     </row>
@@ -3830,28 +3951,28 @@
       <c r="A48" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="33">
+      <c r="C48" s="32">
         <v>1317</v>
       </c>
-      <c r="D48" s="33">
+      <c r="D48" s="32">
         <v>2130</v>
       </c>
-      <c r="E48" s="33">
+      <c r="E48" s="32">
         <v>2141</v>
       </c>
-      <c r="F48" s="32">
+      <c r="F48" s="30">
         <v>2141</v>
       </c>
-      <c r="G48" s="32">
+      <c r="G48" s="30">
         <v>2141</v>
       </c>
-      <c r="H48" s="32">
+      <c r="H48" s="30">
         <v>2141</v>
       </c>
-      <c r="I48" s="32">
+      <c r="I48" s="30">
         <v>2141</v>
       </c>
-      <c r="J48" s="32">
+      <c r="J48" s="30">
         <v>2141</v>
       </c>
     </row>
@@ -3859,28 +3980,28 @@
       <c r="A49" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C49" s="33">
+      <c r="C49" s="32">
         <v>866</v>
       </c>
-      <c r="D49" s="33">
+      <c r="D49" s="32">
         <v>1794</v>
       </c>
-      <c r="E49" s="33">
+      <c r="E49" s="32">
         <v>1722</v>
       </c>
-      <c r="F49" s="32">
+      <c r="F49" s="30">
         <v>1722</v>
       </c>
-      <c r="G49" s="32">
+      <c r="G49" s="30">
         <v>1722</v>
       </c>
-      <c r="H49" s="32">
+      <c r="H49" s="30">
         <v>1722</v>
       </c>
-      <c r="I49" s="32">
+      <c r="I49" s="30">
         <v>1722</v>
       </c>
-      <c r="J49" s="32">
+      <c r="J49" s="30">
         <v>1722</v>
       </c>
     </row>
@@ -3888,28 +4009,28 @@
       <c r="A50" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C50" s="33">
+      <c r="C50" s="32">
         <v>414</v>
       </c>
-      <c r="D50" s="33">
+      <c r="D50" s="32">
         <v>235</v>
       </c>
-      <c r="E50" s="33">
+      <c r="E50" s="32">
         <v>215</v>
       </c>
-      <c r="F50" s="32">
+      <c r="F50" s="30">
         <v>215</v>
       </c>
-      <c r="G50" s="32">
+      <c r="G50" s="30">
         <v>215</v>
       </c>
-      <c r="H50" s="32">
+      <c r="H50" s="30">
         <v>215</v>
       </c>
-      <c r="I50" s="32">
+      <c r="I50" s="30">
         <v>215</v>
       </c>
-      <c r="J50" s="32">
+      <c r="J50" s="30">
         <v>215</v>
       </c>
     </row>
@@ -3917,40 +4038,40 @@
       <c r="A51" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C51" s="34">
+      <c r="C51" s="33">
         <v>6150</v>
       </c>
-      <c r="D51" s="34">
+      <c r="D51" s="33">
         <v>10559</v>
       </c>
-      <c r="E51" s="34">
+      <c r="E51" s="33">
         <v>9850</v>
       </c>
-      <c r="F51" s="36">
+      <c r="F51" s="34">
         <f>SUM(F47:F50)</f>
         <v>9850</v>
       </c>
-      <c r="G51" s="36">
-        <f t="shared" ref="G51:J51" si="12">SUM(G47:G50)</f>
+      <c r="G51" s="34">
+        <f t="shared" ref="G51:J51" si="16">SUM(G47:G50)</f>
         <v>9850</v>
       </c>
-      <c r="H51" s="36">
-        <f t="shared" si="12"/>
+      <c r="H51" s="34">
+        <f t="shared" si="16"/>
         <v>9850</v>
       </c>
-      <c r="I51" s="36">
-        <f t="shared" si="12"/>
+      <c r="I51" s="34">
+        <f t="shared" si="16"/>
         <v>9850</v>
       </c>
-      <c r="J51" s="36">
-        <f t="shared" si="12"/>
+      <c r="J51" s="34">
+        <f t="shared" si="16"/>
         <v>9850</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C52" s="33"/>
-      <c r="D52" s="33"/>
-      <c r="E52" s="33"/>
+      <c r="C52" s="32"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="32"/>
       <c r="F52" s="30"/>
       <c r="G52" s="30"/>
       <c r="H52" s="30"/>
@@ -3961,9 +4082,9 @@
       <c r="A53" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C53" s="33"/>
-      <c r="D53" s="33"/>
-      <c r="E53" s="33"/>
+      <c r="C53" s="32"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
       <c r="F53" s="30"/>
       <c r="G53" s="30"/>
       <c r="H53" s="30"/>
@@ -3974,9 +4095,9 @@
       <c r="A54" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C54" s="33"/>
-      <c r="D54" s="33"/>
-      <c r="E54" s="33"/>
+      <c r="C54" s="32"/>
+      <c r="D54" s="32"/>
+      <c r="E54" s="32"/>
       <c r="F54" s="30"/>
       <c r="G54" s="30"/>
       <c r="H54" s="30"/>
@@ -3987,28 +4108,28 @@
       <c r="A55" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C55" s="33">
+      <c r="C55" s="32">
         <v>713</v>
       </c>
-      <c r="D55" s="33">
+      <c r="D55" s="32">
         <v>1959</v>
       </c>
-      <c r="E55" s="33">
+      <c r="E55" s="32">
         <v>2455</v>
       </c>
-      <c r="F55" s="37">
+      <c r="F55" s="35">
         <v>2455</v>
       </c>
-      <c r="G55" s="37">
+      <c r="G55" s="35">
         <v>2455</v>
       </c>
-      <c r="H55" s="37">
+      <c r="H55" s="35">
         <v>2455</v>
       </c>
-      <c r="I55" s="37">
+      <c r="I55" s="35">
         <v>2455</v>
       </c>
-      <c r="J55" s="37">
+      <c r="J55" s="35">
         <v>2455</v>
       </c>
     </row>
@@ -4016,13 +4137,13 @@
       <c r="A56" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C56" s="33">
+      <c r="C56" s="32">
         <v>2426</v>
       </c>
-      <c r="D56" s="33">
+      <c r="D56" s="32">
         <v>3956</v>
       </c>
-      <c r="E56" s="33">
+      <c r="E56" s="32">
         <v>4164</v>
       </c>
       <c r="F56" s="31">
@@ -4050,28 +4171,28 @@
       <c r="A57" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C57" s="33">
+      <c r="C57" s="32">
         <v>12697</v>
       </c>
-      <c r="D57" s="33">
+      <c r="D57" s="32">
         <v>16969</v>
       </c>
-      <c r="E57" s="33">
+      <c r="E57" s="32">
         <v>18138</v>
       </c>
-      <c r="F57" s="37">
+      <c r="F57" s="35">
         <v>18138</v>
       </c>
-      <c r="G57" s="37">
+      <c r="G57" s="35">
         <v>18138</v>
       </c>
-      <c r="H57" s="37">
+      <c r="H57" s="35">
         <v>18138</v>
       </c>
-      <c r="I57" s="37">
+      <c r="I57" s="35">
         <v>18138</v>
       </c>
-      <c r="J57" s="37">
+      <c r="J57" s="35">
         <v>18138</v>
       </c>
     </row>
@@ -4079,28 +4200,28 @@
       <c r="A58" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C58" s="33">
+      <c r="C58" s="32">
         <v>7609</v>
       </c>
-      <c r="D58" s="33">
+      <c r="D58" s="32">
         <v>10539</v>
       </c>
-      <c r="E58" s="33">
+      <c r="E58" s="32">
         <v>11765</v>
       </c>
-      <c r="F58" s="37">
+      <c r="F58" s="35">
         <v>11765</v>
       </c>
-      <c r="G58" s="37">
+      <c r="G58" s="35">
         <v>11765</v>
       </c>
-      <c r="H58" s="37">
+      <c r="H58" s="35">
         <v>11765</v>
       </c>
-      <c r="I58" s="37">
+      <c r="I58" s="35">
         <v>11765</v>
       </c>
-      <c r="J58" s="37">
+      <c r="J58" s="35">
         <v>11765</v>
       </c>
     </row>
@@ -4108,32 +4229,32 @@
       <c r="A59" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C59" s="33">
+      <c r="C59" s="32">
         <v>1163</v>
       </c>
-      <c r="D59" s="33">
+      <c r="D59" s="32">
         <v>1796</v>
       </c>
-      <c r="E59" s="33">
+      <c r="E59" s="32">
         <v>1475</v>
       </c>
-      <c r="F59" s="37">
+      <c r="F59" s="35">
         <f>IS!F5*Assumptions!F26</f>
         <v>1743.9930000000002</v>
       </c>
-      <c r="G59" s="37">
+      <c r="G59" s="35">
         <f>IS!G5*Assumptions!G26</f>
         <v>1866.0725100000002</v>
       </c>
-      <c r="H59" s="37">
+      <c r="H59" s="35">
         <f>IS!H5*Assumptions!H26</f>
         <v>1992.9654406800003</v>
       </c>
-      <c r="I59" s="37">
+      <c r="I59" s="35">
         <f>IS!I5*Assumptions!I26</f>
         <v>2122.5081943242003</v>
       </c>
-      <c r="J59" s="37">
+      <c r="J59" s="35">
         <f>IS!J5*Assumptions!J26</f>
         <v>2260.4712269552729</v>
       </c>
@@ -4142,28 +4263,28 @@
       <c r="A60" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C60" s="33">
+      <c r="C60" s="32">
         <v>2834</v>
       </c>
-      <c r="D60" s="33">
+      <c r="D60" s="32">
         <v>3585</v>
       </c>
-      <c r="E60" s="33">
+      <c r="E60" s="32">
         <v>4853</v>
       </c>
-      <c r="F60" s="37">
+      <c r="F60" s="35">
         <v>4853</v>
       </c>
-      <c r="G60" s="37">
+      <c r="G60" s="35">
         <v>4853</v>
       </c>
-      <c r="H60" s="37">
+      <c r="H60" s="35">
         <v>4853</v>
       </c>
-      <c r="I60" s="37">
+      <c r="I60" s="35">
         <v>4853</v>
       </c>
-      <c r="J60" s="37">
+      <c r="J60" s="35">
         <v>4853</v>
       </c>
     </row>
@@ -4171,40 +4292,40 @@
       <c r="A61" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C61" s="34">
+      <c r="C61" s="33">
         <v>27442</v>
       </c>
-      <c r="D61" s="34">
+      <c r="D61" s="33">
         <v>38794</v>
       </c>
-      <c r="E61" s="34">
+      <c r="E61" s="33">
         <v>42850</v>
       </c>
-      <c r="F61" s="36">
+      <c r="F61" s="34">
         <f>SUM(F55:F60)</f>
         <v>43492.332397260281</v>
       </c>
-      <c r="G61" s="36">
-        <f t="shared" ref="G61:J61" si="13">SUM(G55:G60)</f>
+      <c r="G61" s="34">
+        <f t="shared" ref="G61:J61" si="17">SUM(G55:G60)</f>
         <v>43932.02566506849</v>
       </c>
-      <c r="H61" s="36">
-        <f t="shared" si="13"/>
+      <c r="H61" s="34">
+        <f t="shared" si="17"/>
         <v>43956.964579492058</v>
       </c>
-      <c r="I61" s="36">
-        <f t="shared" si="13"/>
+      <c r="I61" s="34">
+        <f t="shared" si="17"/>
         <v>44395.452277159042</v>
       </c>
-      <c r="J61" s="36">
-        <f t="shared" si="13"/>
+      <c r="J61" s="34">
+        <f t="shared" si="17"/>
         <v>44862.44167517437</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C62" s="33"/>
-      <c r="D62" s="33"/>
-      <c r="E62" s="33"/>
+      <c r="C62" s="32"/>
+      <c r="D62" s="32"/>
+      <c r="E62" s="32"/>
       <c r="F62" s="30"/>
       <c r="G62" s="30"/>
       <c r="H62" s="30"/>
@@ -4215,37 +4336,37 @@
       <c r="A63" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C63" s="34">
-        <f t="shared" ref="C63:E63" si="14">C41+C51+C61</f>
+      <c r="C63" s="33">
+        <f t="shared" ref="C63:E63" si="18">C41+C51+C61</f>
         <v>101337</v>
       </c>
-      <c r="D63" s="34">
-        <f t="shared" si="14"/>
+      <c r="D63" s="33">
+        <f t="shared" si="18"/>
         <v>137814</v>
       </c>
-      <c r="E63" s="34">
-        <f t="shared" si="14"/>
+      <c r="E63" s="33">
+        <f t="shared" si="18"/>
         <v>148903</v>
       </c>
-      <c r="F63" s="36">
+      <c r="F63" s="34">
         <f>F41+F51+F61</f>
         <v>160771.90704606028</v>
       </c>
-      <c r="G63" s="36">
-        <f t="shared" ref="G63:J63" si="15">G41+G51+G61</f>
-        <v>195667.20003234851</v>
-      </c>
-      <c r="H63" s="36">
-        <f t="shared" si="15"/>
-        <v>232634.21295783768</v>
-      </c>
-      <c r="I63" s="36">
-        <f t="shared" si="15"/>
-        <v>272416.00947728951</v>
-      </c>
-      <c r="J63" s="36">
-        <f t="shared" si="15"/>
-        <v>314783.62277050572</v>
+      <c r="G63" s="34">
+        <f t="shared" ref="G63:J63" si="19">G41+G51+G61</f>
+        <v>173271.0602153365</v>
+      </c>
+      <c r="H63" s="34">
+        <f t="shared" si="19"/>
+        <v>186225.72503363303</v>
+      </c>
+      <c r="I63" s="34">
+        <f t="shared" si="19"/>
+        <v>200434.37081892474</v>
+      </c>
+      <c r="J63" s="34">
+        <f t="shared" si="19"/>
+        <v>215566.57858026036</v>
       </c>
     </row>
   </sheetData>
@@ -4258,23 +4379,23 @@
   <sheetPr>
     <tabColor theme="2" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="64.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -4288,27 +4409,62 @@
       <c r="E4" s="5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F4" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="36">
         <v>23268</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="36">
         <v>26248</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="36">
         <v>26750</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F7" s="31">
+        <f>IS!F27</f>
+        <v>32075.927567999999</v>
+      </c>
+      <c r="G7" s="31">
+        <f>IS!G27</f>
+        <v>34455.599718480007</v>
+      </c>
+      <c r="H7" s="31">
+        <f>IS!H27</f>
+        <v>36942.074011065604</v>
+      </c>
+      <c r="I7" s="31">
+        <f>IS!I27</f>
+        <v>39343.308821784864</v>
+      </c>
+      <c r="J7" s="31">
+        <f>IS!J27</f>
+        <v>41900.623895200879</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>67</v>
       </c>
@@ -4316,7 +4472,7 @@
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -4329,8 +4485,28 @@
       <c r="E9" s="6">
         <v>4812</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F9" s="22">
+        <f>'PP&amp;E Sch'!F11</f>
+        <v>2659.65</v>
+      </c>
+      <c r="G9" s="22">
+        <f>'PP&amp;E Sch'!G11</f>
+        <v>2867.1851670000001</v>
+      </c>
+      <c r="H9" s="22">
+        <f>'PP&amp;E Sch'!H11</f>
+        <v>3089.2477956900002</v>
+      </c>
+      <c r="I9" s="22">
+        <f>'PP&amp;E Sch'!I11</f>
+        <v>3334.8807862538106</v>
+      </c>
+      <c r="J9" s="22">
+        <f>'PP&amp;E Sch'!J11</f>
+        <v>3600.0881851346194</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>125</v>
       </c>
@@ -4343,8 +4519,28 @@
       <c r="E10" s="6">
         <v>10858</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10" s="30">
+        <f>IS!F25</f>
+        <v>12473.971832000001</v>
+      </c>
+      <c r="G10" s="30">
+        <f>IS!G25</f>
+        <v>13399.399890520002</v>
+      </c>
+      <c r="H10" s="30">
+        <f>IS!H25</f>
+        <v>14366.362115414402</v>
+      </c>
+      <c r="I10" s="30">
+        <f>IS!I25</f>
+        <v>15300.175652916338</v>
+      </c>
+      <c r="J10" s="30">
+        <f>IS!J25</f>
+        <v>16294.687070355898</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>126</v>
       </c>
@@ -4358,7 +4554,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -4372,7 +4568,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>69</v>
       </c>
@@ -4386,7 +4582,7 @@
         <v>-2570</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>70</v>
       </c>
@@ -4400,7 +4596,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>71</v>
       </c>
@@ -4414,7 +4610,7 @@
         <v>-110</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>72</v>
       </c>
@@ -4428,7 +4624,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>73</v>
       </c>
@@ -4442,7 +4638,7 @@
         <v>-327</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>74</v>
       </c>
@@ -4456,12 +4652,12 @@
         <v>833</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>75</v>
       </c>
@@ -4469,7 +4665,7 @@
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>76</v>
       </c>
@@ -4482,8 +4678,28 @@
       <c r="E21" s="6">
         <v>-1769</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" s="30">
+        <f>-('WC Sch'!F5-'WC Sch'!E5)</f>
+        <v>-2288.4410958904118</v>
+      </c>
+      <c r="G21" s="30">
+        <f>-('WC Sch'!G5-'WC Sch'!F5)</f>
+        <v>-1829.9981342465762</v>
+      </c>
+      <c r="H21" s="30">
+        <f>-('WC Sch'!H5-'WC Sch'!G5)</f>
+        <v>-2398.7978676493149</v>
+      </c>
+      <c r="I21" s="30">
+        <f>-('WC Sch'!I5-'WC Sch'!H5)</f>
+        <v>-1867.3813170207141</v>
+      </c>
+      <c r="J21" s="30">
+        <f>-('WC Sch'!J5-'WC Sch'!I5)</f>
+        <v>-2570.2701969624541</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -4497,7 +4713,7 @@
         <v>-1024</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -4510,8 +4726,28 @@
       <c r="E23" s="6">
         <v>176</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" s="30">
+        <f>'WC Sch'!F6-'WC Sch'!E6</f>
+        <v>373.33939726027438</v>
+      </c>
+      <c r="G23" s="30">
+        <f>'WC Sch'!G6-'WC Sch'!F6</f>
+        <v>317.61375780821982</v>
+      </c>
+      <c r="H23" s="30">
+        <f>'WC Sch'!H6-'WC Sch'!G6</f>
+        <v>-101.95401625643717</v>
+      </c>
+      <c r="I23" s="30">
+        <f>'WC Sch'!I6-'WC Sch'!H6</f>
+        <v>308.94494402278178</v>
+      </c>
+      <c r="J23" s="30">
+        <f>'WC Sch'!J6-'WC Sch'!I6</f>
+        <v>329.02636538426395</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -4524,13 +4760,33 @@
       <c r="E24" s="6">
         <v>2322</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" s="30">
+        <f>SUM(BS!F57:F59)-SUM(BS!E57:E59)</f>
+        <v>268.99299999999857</v>
+      </c>
+      <c r="G24" s="30">
+        <f>SUM(BS!G57:G59)-SUM(BS!F57:F59)</f>
+        <v>122.07951000000321</v>
+      </c>
+      <c r="H24" s="30">
+        <f>SUM(BS!H57:H59)-SUM(BS!G57:G59)</f>
+        <v>126.89293067999824</v>
+      </c>
+      <c r="I24" s="30">
+        <f>SUM(BS!I57:I59)-SUM(BS!H57:H59)</f>
+        <v>129.54275364420027</v>
+      </c>
+      <c r="J24" s="30">
+        <f>SUM(BS!J57:J59)-SUM(BS!I57:I59)</f>
+        <v>137.96303263107256</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>79</v>
       </c>
@@ -4543,8 +4799,28 @@
       <c r="E26" s="11">
         <v>41296</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" s="34">
+        <f>SUM(F7:F18,F21:F24)</f>
+        <v>45563.440701369866</v>
+      </c>
+      <c r="G26" s="34">
+        <f t="shared" ref="G26:J26" si="0">SUM(G7:G18,G21:G24)</f>
+        <v>49331.879909561656</v>
+      </c>
+      <c r="H26" s="34">
+        <f t="shared" si="0"/>
+        <v>52023.824968944253</v>
+      </c>
+      <c r="I26" s="34">
+        <f t="shared" si="0"/>
+        <v>56549.471641601282</v>
+      </c>
+      <c r="J26" s="34">
+        <f t="shared" si="0"/>
+        <v>59692.118351744277</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>80</v>
       </c>
@@ -4557,8 +4833,28 @@
       <c r="E27" s="6">
         <v>-5602</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" s="30">
+        <f>-IS!F25</f>
+        <v>-12473.971832000001</v>
+      </c>
+      <c r="G27" s="30">
+        <f>-IS!G25</f>
+        <v>-13399.399890520002</v>
+      </c>
+      <c r="H27" s="30">
+        <f>-IS!H25</f>
+        <v>-14366.362115414402</v>
+      </c>
+      <c r="I27" s="30">
+        <f>-IS!I25</f>
+        <v>-15300.175652916338</v>
+      </c>
+      <c r="J27" s="30">
+        <f>-IS!J25</f>
+        <v>-16294.687070355898</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>81</v>
       </c>
@@ -4571,13 +4867,33 @@
       <c r="E28" s="11">
         <v>35694</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F28" s="34">
+        <f>F26+F27</f>
+        <v>33089.468869369863</v>
+      </c>
+      <c r="G28" s="34">
+        <f t="shared" ref="G28:J28" si="1">G26+G27</f>
+        <v>35932.480019041657</v>
+      </c>
+      <c r="H28" s="34">
+        <f t="shared" si="1"/>
+        <v>37657.462853529854</v>
+      </c>
+      <c r="I28" s="34">
+        <f t="shared" si="1"/>
+        <v>41249.295988684942</v>
+      </c>
+      <c r="J28" s="34">
+        <f t="shared" si="1"/>
+        <v>43397.431281388381</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -4589,6 +4905,26 @@
       </c>
       <c r="E32" s="6">
         <v>-2237</v>
+      </c>
+      <c r="F32" s="22">
+        <f>-('PP&amp;E Sch'!F7+(BS!F10-BS!E10))</f>
+        <v>-2360.0672600000003</v>
+      </c>
+      <c r="G32" s="22">
+        <f>-('PP&amp;E Sch'!G7+(BS!G10-BS!F10))</f>
+        <v>-2663.7749082000005</v>
+      </c>
+      <c r="H32" s="22">
+        <f>-('PP&amp;E Sch'!H7+(BS!H10-BS!G10))</f>
+        <v>-2972.9894014818005</v>
+      </c>
+      <c r="I32" s="22">
+        <f>-('PP&amp;E Sch'!I7+(BS!I10-BS!H10))</f>
+        <v>-3189.1731926577459</v>
+      </c>
+      <c r="J32" s="22">
+        <f>-('PP&amp;E Sch'!J7+(BS!J10-BS!I10))</f>
+        <v>-3471.8927788658098</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -4809,7 +5145,7 @@
         <v>-73048</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
         <v>100</v>
       </c>
@@ -4823,7 +5159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="8" t="s">
         <v>101</v>
       </c>
@@ -4837,7 +5173,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="8" t="s">
         <v>102</v>
       </c>
@@ -4851,7 +5187,7 @@
         <v>-6403</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="8" t="s">
         <v>103</v>
       </c>
@@ -4865,7 +5201,7 @@
         <v>-6978</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="8" t="s">
         <v>104</v>
       </c>
@@ -4879,7 +5215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="8" t="s">
         <v>105</v>
       </c>
@@ -4893,7 +5229,7 @@
         <v>-3240</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="8" t="s">
         <v>106</v>
       </c>
@@ -4907,7 +5243,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>97</v>
       </c>
@@ -4915,7 +5251,7 @@
       <c r="D56" s="7"/>
       <c r="E56" s="7"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="8" t="s">
         <v>107</v>
       </c>
@@ -4929,7 +5265,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="8" t="s">
         <v>99</v>
       </c>
@@ -4943,7 +5279,7 @@
         <v>73987</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="8" t="s">
         <v>108</v>
       </c>
@@ -4957,7 +5293,7 @@
         <v>2591</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="8" t="s">
         <v>109</v>
       </c>
@@ -4971,7 +5307,7 @@
         <v>6688</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="8" t="s">
         <v>111</v>
       </c>
@@ -4985,7 +5321,7 @@
         <v>7735</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="8" t="s">
         <v>110</v>
       </c>
@@ -4999,7 +5335,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="8" t="s">
         <v>106</v>
       </c>
@@ -5013,7 +5349,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>98</v>
       </c>
@@ -5026,13 +5362,33 @@
       <c r="E64" s="11">
         <v>-1946</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F64" s="29">
+        <f>F32</f>
+        <v>-2360.0672600000003</v>
+      </c>
+      <c r="G64" s="29">
+        <f t="shared" ref="G64:J64" si="2">G32</f>
+        <v>-2663.7749082000005</v>
+      </c>
+      <c r="H64" s="29">
+        <f t="shared" si="2"/>
+        <v>-2972.9894014818005</v>
+      </c>
+      <c r="I64" s="29">
+        <f t="shared" si="2"/>
+        <v>-3189.1731926577459</v>
+      </c>
+      <c r="J64" s="29">
+        <f t="shared" si="2"/>
+        <v>-3471.8927788658098</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C65" s="7"/>
       <c r="D65" s="7"/>
       <c r="E65" s="7"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="13" t="s">
         <v>112</v>
       </c>
@@ -5040,12 +5396,12 @@
       <c r="D66" s="7"/>
       <c r="E66" s="7"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
       <c r="E67" s="7"/>
     </row>
-    <row r="68" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="10" t="s">
         <v>114</v>
       </c>
@@ -5059,7 +5415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>113</v>
       </c>
@@ -5073,7 +5429,7 @@
         <v>-2355</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>115</v>
       </c>
@@ -5087,7 +5443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>86</v>
       </c>
@@ -5101,7 +5457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>116</v>
       </c>
@@ -5115,7 +5471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>117</v>
       </c>
@@ -5128,8 +5484,28 @@
       <c r="E73" s="6">
         <v>-20287</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F73" s="18">
+        <f>-(IS!F27*Assumptions!F22)</f>
+        <v>-20849.352919199999</v>
+      </c>
+      <c r="G73" s="18">
+        <f>-(IS!G27*Assumptions!G22)</f>
+        <v>-22396.139817012005</v>
+      </c>
+      <c r="H73" s="18">
+        <f>-(IS!H27*Assumptions!H22)</f>
+        <v>-24012.348107192644</v>
+      </c>
+      <c r="I73" s="18">
+        <f>-(IS!I27*Assumptions!I22)</f>
+        <v>-25573.150734160161</v>
+      </c>
+      <c r="J73" s="18">
+        <f>-(IS!J27*Assumptions!J22)</f>
+        <v>-27235.405531880573</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>118</v>
       </c>
@@ -5142,13 +5518,33 @@
       <c r="E74" s="11">
         <v>-24161</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F74">
+        <f>SUM(F68:F73)</f>
+        <v>-20849.352919199999</v>
+      </c>
+      <c r="G74">
+        <f t="shared" ref="G74:J74" si="3">SUM(G68:G73)</f>
+        <v>-22396.139817012005</v>
+      </c>
+      <c r="H74">
+        <f t="shared" si="3"/>
+        <v>-24012.348107192644</v>
+      </c>
+      <c r="I74">
+        <f t="shared" si="3"/>
+        <v>-25573.150734160161</v>
+      </c>
+      <c r="J74">
+        <f t="shared" si="3"/>
+        <v>-27235.405531880573</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>119</v>
       </c>
@@ -5161,8 +5557,28 @@
       <c r="E76" s="6">
         <v>9587</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F76" s="30">
+        <f>SUM(F28,F64,F74)</f>
+        <v>9880.0486901698641</v>
+      </c>
+      <c r="G76" s="30">
+        <f t="shared" ref="G76:J76" si="4">SUM(G28,G64,G74)</f>
+        <v>10872.565293829652</v>
+      </c>
+      <c r="H76" s="30">
+        <f t="shared" si="4"/>
+        <v>10672.125344855413</v>
+      </c>
+      <c r="I76" s="30">
+        <f t="shared" si="4"/>
+        <v>12486.972061867033</v>
+      </c>
+      <c r="J76" s="30">
+        <f t="shared" si="4"/>
+        <v>12690.132970641997</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>120</v>
       </c>
@@ -5176,7 +5592,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>121</v>
       </c>
@@ -5189,8 +5605,28 @@
       <c r="E78" s="6">
         <v>14786</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F78" s="37">
+        <f>E79</f>
+        <v>24455</v>
+      </c>
+      <c r="G78" s="37">
+        <f t="shared" ref="G78:J78" si="5">F79</f>
+        <v>34335.04869016986</v>
+      </c>
+      <c r="H78" s="37">
+        <f t="shared" si="5"/>
+        <v>45207.613983999516</v>
+      </c>
+      <c r="I78" s="37">
+        <f t="shared" si="5"/>
+        <v>55879.739328854928</v>
+      </c>
+      <c r="J78" s="37">
+        <f t="shared" si="5"/>
+        <v>68366.711390721961</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>122</v>
       </c>
@@ -5203,8 +5639,28 @@
       <c r="E79" s="6">
         <v>24455</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F79" s="30">
+        <f>SUM(F76,F78)</f>
+        <v>34335.04869016986</v>
+      </c>
+      <c r="G79" s="30">
+        <f t="shared" ref="G79:J79" si="6">SUM(G76,G78)</f>
+        <v>45207.613983999516</v>
+      </c>
+      <c r="H79" s="30">
+        <f t="shared" si="6"/>
+        <v>55879.739328854928</v>
+      </c>
+      <c r="I79" s="30">
+        <f t="shared" si="6"/>
+        <v>68366.711390721961</v>
+      </c>
+      <c r="J79" s="30">
+        <f t="shared" si="6"/>
+        <v>81056.844361363954</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="s">
         <v>123</v>
       </c>
@@ -5232,56 +5688,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90E68197-B81D-A946-87FA-197633624652}">
-  <sheetPr>
-    <tabColor theme="2" tint="-0.249977111117893"/>
-  </sheetPr>
-  <dimension ref="A2:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C3">
-        <f>BS!C45-(BS!C70+BS!C80)</f>
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <f>BS!D45-(BS!D70+BS!D80)</f>
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <f>BS!E45-(BS!E70+BS!E80)</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="C3:E3">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5811CD45-A520-A542-A284-F1CD7853A834}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -5332,42 +5738,37 @@
         <v>173</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>178</v>
-      </c>
-    </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C6" s="29"/>
       <c r="D6" s="29"/>
       <c r="E6" s="29"/>
       <c r="F6" s="29">
         <f>E8</f>
-        <v>27629</v>
+        <v>31290</v>
       </c>
       <c r="G6" s="29">
         <f t="shared" ref="G6:J6" si="0">F8</f>
-        <v>30070.590199999999</v>
+        <v>33731.590199999999</v>
       </c>
       <c r="H6" s="29">
         <f t="shared" si="0"/>
-        <v>32683.091713999998</v>
+        <v>36344.091714000002</v>
       </c>
       <c r="I6" s="29">
         <f t="shared" si="0"/>
-        <v>35572.891602985997</v>
+        <v>39233.891602986005</v>
       </c>
       <c r="J6" s="29">
         <f t="shared" si="0"/>
-        <v>38692.978648642573</v>
+        <v>42353.97864864258</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C7" s="29"/>
       <c r="D7" s="29"/>
@@ -5395,42 +5796,42 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>179</v>
-      </c>
-      <c r="C8" s="29">
-        <v>26709</v>
-      </c>
-      <c r="D8" s="29">
-        <v>27240</v>
-      </c>
-      <c r="E8" s="29">
-        <v>27629</v>
+        <v>178</v>
+      </c>
+      <c r="C8" s="40">
+        <v>30089</v>
+      </c>
+      <c r="D8" s="40">
+        <v>30587</v>
+      </c>
+      <c r="E8" s="40">
+        <v>31290</v>
       </c>
       <c r="F8" s="29">
         <f>(F7)+F6</f>
-        <v>30070.590199999999</v>
+        <v>33731.590199999999</v>
       </c>
       <c r="G8" s="29">
         <f t="shared" ref="G8:J8" si="1">(G7)+G6</f>
-        <v>32683.091713999998</v>
+        <v>36344.091714000002</v>
       </c>
       <c r="H8" s="29">
         <f t="shared" si="1"/>
-        <v>35572.891602985997</v>
+        <v>39233.891602986005</v>
       </c>
       <c r="I8" s="29">
         <f t="shared" si="1"/>
-        <v>38692.978648642573</v>
+        <v>42353.97864864258</v>
       </c>
       <c r="J8" s="29">
         <f t="shared" si="1"/>
-        <v>42083.685489075484</v>
+        <v>45744.685489075491</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
       <c r="F9" s="29"/>
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
@@ -5439,92 +5840,92 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>184</v>
-      </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
+        <v>183</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
       <c r="F10" s="29">
         <f>E12</f>
-        <v>17559</v>
+        <v>19512</v>
       </c>
       <c r="G10" s="29">
         <f t="shared" ref="G10:J10" si="2">F12</f>
-        <v>19907.465</v>
+        <v>22171.65</v>
       </c>
       <c r="H10" s="29">
         <f t="shared" si="2"/>
-        <v>22463.465167000002</v>
+        <v>25038.835167000001</v>
       </c>
       <c r="I10" s="29">
         <f t="shared" si="2"/>
-        <v>25241.527962690001</v>
+        <v>28128.082962690001</v>
       </c>
       <c r="J10" s="29">
         <f t="shared" si="2"/>
-        <v>28265.223748943812</v>
+        <v>31462.96374894381</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>185</v>
-      </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
+        <v>184</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
       <c r="F11" s="29">
         <f>F6*Assumptions!F20</f>
-        <v>2348.4650000000001</v>
+        <v>2659.65</v>
       </c>
       <c r="G11" s="29">
         <f>G6*Assumptions!G20</f>
-        <v>2556.0001670000001</v>
+        <v>2867.1851670000001</v>
       </c>
       <c r="H11" s="29">
         <f>H6*Assumptions!H20</f>
-        <v>2778.0627956900003</v>
+        <v>3089.2477956900002</v>
       </c>
       <c r="I11" s="29">
         <f>I6*Assumptions!I20</f>
-        <v>3023.6957862538102</v>
+        <v>3334.8807862538106</v>
       </c>
       <c r="J11" s="29">
         <f>J6*Assumptions!J20</f>
-        <v>3288.903185134619</v>
+        <v>3600.0881851346194</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>180</v>
-      </c>
-      <c r="C12" s="29">
-        <v>15053</v>
-      </c>
-      <c r="D12" s="29">
-        <v>16427</v>
-      </c>
-      <c r="E12" s="29">
-        <v>17559</v>
+        <v>179</v>
+      </c>
+      <c r="C12" s="40">
+        <v>16743</v>
+      </c>
+      <c r="D12" s="40">
+        <v>18217</v>
+      </c>
+      <c r="E12" s="40">
+        <v>19512</v>
       </c>
       <c r="F12" s="29">
         <f>F10+F11</f>
-        <v>19907.465</v>
+        <v>22171.65</v>
       </c>
       <c r="G12" s="29">
         <f t="shared" ref="G12:J12" si="3">G10+G11</f>
-        <v>22463.465167000002</v>
+        <v>25038.835167000001</v>
       </c>
       <c r="H12" s="29">
         <f t="shared" si="3"/>
-        <v>25241.527962690001</v>
+        <v>28128.082962690001</v>
       </c>
       <c r="I12" s="29">
         <f t="shared" si="3"/>
-        <v>28265.223748943812</v>
+        <v>31462.96374894381</v>
       </c>
       <c r="J12" s="29">
         <f t="shared" si="3"/>
-        <v>31554.126934078431</v>
+        <v>35063.05193407843</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -5539,39 +5940,39 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C14" s="29">
         <f t="shared" ref="C14:D14" si="4">C8-C12</f>
-        <v>11656</v>
+        <v>13346</v>
       </c>
       <c r="D14" s="29">
         <f t="shared" si="4"/>
-        <v>10813</v>
+        <v>12370</v>
       </c>
       <c r="E14" s="29">
         <f>E8-E12</f>
-        <v>10070</v>
+        <v>11778</v>
       </c>
       <c r="F14" s="29">
         <f>F8-F12</f>
-        <v>10163.125199999999</v>
+        <v>11559.940199999997</v>
       </c>
       <c r="G14" s="29">
         <f t="shared" ref="G14:J14" si="5">G8-G12</f>
-        <v>10219.626546999996</v>
+        <v>11305.256547000001</v>
       </c>
       <c r="H14" s="29">
         <f t="shared" si="5"/>
-        <v>10331.363640295996</v>
+        <v>11105.808640296003</v>
       </c>
       <c r="I14" s="29">
         <f t="shared" si="5"/>
-        <v>10427.754899698761</v>
+        <v>10891.01489969877</v>
       </c>
       <c r="J14" s="29">
         <f t="shared" si="5"/>
-        <v>10529.558554997053</v>
+        <v>10681.633554997061</v>
       </c>
     </row>
   </sheetData>
@@ -5579,7 +5980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F628F37-A227-084E-9F65-67CF215B7A7C}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -5594,7 +5995,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -5629,7 +6030,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C5" s="30">
         <f>Assumptions!C11/365*IS!C5</f>
@@ -5666,7 +6067,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C6" s="30">
         <f>Assumptions!C12/365*IS!C19</f>
@@ -5703,7 +6104,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C7" s="30">
         <f>Assumptions!C13/365</f>
@@ -5743,11 +6144,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA9760A0-4F56-4945-A987-A29095672D87}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD350CFE-D0BB-9A48-980A-212CF0B3318D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Phase 5: WACC and UFCF
</commit_message>
<xml_diff>
--- a/model/3 statement model .xlsx
+++ b/model/3 statement model .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ravishagosain/Desktop/WorkX/Finance/projects/3 statement model/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F114AF10-D75F-2E42-A8D8-2EF5703215AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80AFD6E4-DBAC-8745-9871-6BDCC6EA2D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="11" xr2:uid="{C2ABDD43-7712-494D-BFB8-6BE793A7A1EB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="8" xr2:uid="{C2ABDD43-7712-494D-BFB8-6BE793A7A1EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,8 @@
     <sheet name="CFS" sheetId="5" r:id="rId5"/>
     <sheet name="PP&amp;E Sch" sheetId="7" r:id="rId6"/>
     <sheet name="WC Sch" sheetId="8" r:id="rId7"/>
-    <sheet name="Sheet1" sheetId="12" r:id="rId8"/>
-    <sheet name="WACC" sheetId="9" r:id="rId9"/>
+    <sheet name="WACC" sheetId="9" r:id="rId8"/>
+    <sheet name="UFCF" sheetId="12" r:id="rId9"/>
     <sheet name="DCF" sheetId="10" r:id="rId10"/>
     <sheet name="Sensitivity" sheetId="11" r:id="rId11"/>
     <sheet name="Check" sheetId="6" r:id="rId12"/>
@@ -45,8 +45,85 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Microsoft Office User</author>
+  </authors>
+  <commentList>
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{BA0E1620-C34A-C14C-A474-1B186F6E8C69}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">Source: Reuters, “Indian rupee, bonds to track oil prices; local and US inflation data in focus,” August 10, 2026. 10-year India benchmark government bond yield reported at 6.7651% during the prior week.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>https://www.reuters.com/world/india/indian-rupee-bonds-track-oil-prices-local-us-inflation-data-focus-2026-08-10/?</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{731D647D-038C-014A-93A0-0C2968DBF2FA}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Source: Yahoo Finance, Infosys Limited (INFY), Beta (5Y Monthly), accessed August 16, 2026.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{74BA8932-0107-FB44-8E49-3611279AA554}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Source: Aswath Damodaran, NYU Stern, Country Equity Risk Premiums, India. Total Equity Risk Premium = 7.27%. Data updated January 2026.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0" xr:uid="{749C2E35-9546-B142-AAB0-806C75177128}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Source: Current Infosys market capitalization from NSE/Yahoo Finance, accessed August 2026.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="213">
   <si>
     <t>Infosys Limited</t>
   </si>
@@ -625,16 +702,78 @@
   </si>
   <si>
     <t>WC Schedule (₹ Crores)</t>
+  </si>
+  <si>
+    <t>WACC</t>
+  </si>
+  <si>
+    <t>Risk free rate</t>
+  </si>
+  <si>
+    <t>Beta</t>
+  </si>
+  <si>
+    <t>Equity Risk Premium (ERP)</t>
+  </si>
+  <si>
+    <t>Cost of Equity</t>
+  </si>
+  <si>
+    <t>Total Debt</t>
+  </si>
+  <si>
+    <t>Interest Expense</t>
+  </si>
+  <si>
+    <t>Cost of debt (pre tax)</t>
+  </si>
+  <si>
+    <t>Tax rate</t>
+  </si>
+  <si>
+    <t>Cost of debt (after tax)</t>
+  </si>
+  <si>
+    <t>Market Cap</t>
+  </si>
+  <si>
+    <t>Weight of Equity</t>
+  </si>
+  <si>
+    <t>Weight of Debt</t>
+  </si>
+  <si>
+    <t>Unlevered Free Cash Flow (₹ Crores)</t>
+  </si>
+  <si>
+    <t>Tax Rate</t>
+  </si>
+  <si>
+    <t>NOPAT</t>
+  </si>
+  <si>
+    <t>D&amp;A</t>
+  </si>
+  <si>
+    <t>Change in NWC</t>
+  </si>
+  <si>
+    <t>UFCF</t>
+  </si>
+  <si>
+    <t>UFCF Growth%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\)"/>
+    <numFmt numFmtId="168" formatCode="0.0000%"/>
+    <numFmt numFmtId="169" formatCode="0.000000%"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -703,6 +842,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -745,7 +898,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -807,6 +960,11 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1150,9 +1308,7 @@
   <cols>
     <col min="1" max="16384" width="12.83203125" style="2"/>
   </cols>
-  <sheetData>
-    <row r="1" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6145,19 +6301,467 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA9760A0-4F56-4945-A987-A29095672D87}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD350CFE-D0BB-9A48-980A-212CF0B3318D}">
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="41" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" s="42">
+        <v>6.7651000000000003E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B4" s="7">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B5" s="27">
+        <v>7.2700000000000001E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="44">
+        <f>B3+B4*B5</f>
+        <v>7.7102000000000004E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="31">
+        <f>BS!E47+BS!E55</f>
+        <v>8227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="18">
+        <f>IS!E17</f>
+        <v>416</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B10" s="43">
+        <f>B9/B8</f>
+        <v>5.0565212106478664E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" s="19">
+        <f>Assumptions!F18</f>
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>202</v>
+      </c>
+      <c r="B12" s="43">
+        <f>B10*(1-B11)</f>
+        <v>3.6406952716664637E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" s="45">
+        <v>620000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>204</v>
+      </c>
+      <c r="B15" s="43">
+        <f>B14/(B14+B8)</f>
+        <v>0.98690441512383265</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>205</v>
+      </c>
+      <c r="B16" s="43">
+        <f>B8/(B14+B8)</f>
+        <v>1.3095584876167373E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>193</v>
+      </c>
+      <c r="B18" s="43">
+        <f>B15*B6+B16*B12</f>
+        <v>7.6569074554261443E-2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD350CFE-D0BB-9A48-980A-212CF0B3318D}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA9760A0-4F56-4945-A987-A29095672D87}">
+  <sheetPr>
+    <tabColor theme="9" tint="0.39997558519241921"/>
+  </sheetPr>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" s="31">
+        <f>IS!C29</f>
+        <v>31800</v>
+      </c>
+      <c r="D5" s="31">
+        <f>IS!D29</f>
+        <v>36458</v>
+      </c>
+      <c r="E5" s="31">
+        <f>IS!E29</f>
+        <v>38024</v>
+      </c>
+      <c r="F5" s="31">
+        <f>IS!F29</f>
+        <v>40635.036900000006</v>
+      </c>
+      <c r="G5" s="31">
+        <f>IS!G29</f>
+        <v>43666.096734000006</v>
+      </c>
+      <c r="H5" s="31">
+        <f>IS!H29</f>
+        <v>46834.687855980002</v>
+      </c>
+      <c r="I5" s="31">
+        <f>IS!I29</f>
+        <v>49878.942566618702</v>
+      </c>
+      <c r="J5" s="31">
+        <f>IS!J29</f>
+        <v>53121.073833448914</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C6" s="19">
+        <f>Assumptions!C18</f>
+        <v>0.2646714913250956</v>
+      </c>
+      <c r="D6" s="19">
+        <f>Assumptions!D18</f>
+        <v>0.27064577081249308</v>
+      </c>
+      <c r="E6" s="19">
+        <f>Assumptions!E18</f>
+        <v>0.28871516698574773</v>
+      </c>
+      <c r="F6" s="19">
+        <f>Assumptions!F18</f>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="G6" s="19">
+        <f>Assumptions!G18</f>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="H6" s="19">
+        <f>Assumptions!H18</f>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="I6" s="19">
+        <f>Assumptions!I18</f>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="J6" s="19">
+        <f>Assumptions!J18</f>
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7" s="30">
+        <f>C5*(1-C6)</f>
+        <v>23383.446575861959</v>
+      </c>
+      <c r="D7">
+        <f t="shared" ref="D7:J7" si="0">D5*(1-D6)</f>
+        <v>26590.796487718126</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>27045.894490533927</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>29257.226568000002</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>31439.589648480003</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>33720.975256305603</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>35912.838647965465</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>38247.173160083214</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="22">
+        <f>'PP&amp;E Sch'!C11</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="22">
+        <f>'PP&amp;E Sch'!D11</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="22">
+        <f>'PP&amp;E Sch'!E11</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="22">
+        <f>'PP&amp;E Sch'!F11</f>
+        <v>2659.65</v>
+      </c>
+      <c r="G8" s="22">
+        <f>'PP&amp;E Sch'!G11</f>
+        <v>2867.1851670000001</v>
+      </c>
+      <c r="H8" s="22">
+        <f>'PP&amp;E Sch'!H11</f>
+        <v>3089.2477956900002</v>
+      </c>
+      <c r="I8" s="22">
+        <f>'PP&amp;E Sch'!I11</f>
+        <v>3334.8807862538106</v>
+      </c>
+      <c r="J8" s="22">
+        <f>'PP&amp;E Sch'!J11</f>
+        <v>3600.0881851346194</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="22">
+        <f>'PP&amp;E Sch'!C7</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="22">
+        <f>'PP&amp;E Sch'!D7</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="22">
+        <f>'PP&amp;E Sch'!E7</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="22">
+        <f>'PP&amp;E Sch'!F7</f>
+        <v>2441.5902000000001</v>
+      </c>
+      <c r="G9" s="22">
+        <f>'PP&amp;E Sch'!G7</f>
+        <v>2612.5015140000005</v>
+      </c>
+      <c r="H9" s="22">
+        <f>'PP&amp;E Sch'!H7</f>
+        <v>2889.7998889860005</v>
+      </c>
+      <c r="I9" s="22">
+        <f>'PP&amp;E Sch'!I7</f>
+        <v>3120.087045656574</v>
+      </c>
+      <c r="J9" s="22">
+        <f>'PP&amp;E Sch'!J7</f>
+        <v>3390.7068404329093</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>210</v>
+      </c>
+      <c r="C10" s="30"/>
+      <c r="D10" s="31">
+        <f>('WC Sch'!D5+'WC Sch'!D7-'WC Sch'!D6)-('WC Sch'!C5+'WC Sch'!C7-'WC Sch'!C6)</f>
+        <v>7890</v>
+      </c>
+      <c r="E10" s="31">
+        <f>('WC Sch'!E5+'WC Sch'!E7-'WC Sch'!E6)-('WC Sch'!D5+'WC Sch'!D7-'WC Sch'!D6)</f>
+        <v>757</v>
+      </c>
+      <c r="F10" s="31">
+        <f>('WC Sch'!F5+'WC Sch'!F7-'WC Sch'!F6)-('WC Sch'!E5+'WC Sch'!E7-'WC Sch'!E6)</f>
+        <v>1915.1016986301365</v>
+      </c>
+      <c r="G10" s="31">
+        <f>('WC Sch'!G5+'WC Sch'!G7-'WC Sch'!G6)-('WC Sch'!F5+'WC Sch'!F7-'WC Sch'!F6)</f>
+        <v>1512.3843764383564</v>
+      </c>
+      <c r="H10" s="31">
+        <f>('WC Sch'!H5+'WC Sch'!H7-'WC Sch'!H6)-('WC Sch'!G5+'WC Sch'!G7-'WC Sch'!G6)</f>
+        <v>2500.7518839057557</v>
+      </c>
+      <c r="I10" s="31">
+        <f>('WC Sch'!I5+'WC Sch'!I7-'WC Sch'!I6)-('WC Sch'!H5+'WC Sch'!H7-'WC Sch'!H6)</f>
+        <v>1558.4363729979304</v>
+      </c>
+      <c r="J10" s="31">
+        <f>('WC Sch'!J5+'WC Sch'!J7-'WC Sch'!J6)-('WC Sch'!I5+'WC Sch'!I7-'WC Sch'!I6)</f>
+        <v>2241.243831578191</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" s="34">
+        <f>D7+D8-D9-D10</f>
+        <v>18700.796487718126</v>
+      </c>
+      <c r="E12" s="34">
+        <f t="shared" ref="E12:J12" si="1">E7+E8-E9-E10</f>
+        <v>26288.894490533927</v>
+      </c>
+      <c r="F12" s="34">
+        <f t="shared" si="1"/>
+        <v>27560.184669369868</v>
+      </c>
+      <c r="G12" s="34">
+        <f t="shared" si="1"/>
+        <v>30181.888925041651</v>
+      </c>
+      <c r="H12" s="34">
+        <f t="shared" si="1"/>
+        <v>31419.671279103848</v>
+      </c>
+      <c r="I12" s="34">
+        <f t="shared" si="1"/>
+        <v>34569.196015564768</v>
+      </c>
+      <c r="J12" s="34">
+        <f t="shared" si="1"/>
+        <v>36215.310673206732</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>212</v>
+      </c>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43">
+        <f t="shared" ref="E14:F14" si="2">F12/E12-1</f>
+        <v>4.8358449583861596E-2</v>
+      </c>
+      <c r="G14" s="43">
+        <f>G12/F12-1</f>
+        <v>9.5126512653070927E-2</v>
+      </c>
+      <c r="H14" s="43">
+        <f t="shared" ref="H14:J14" si="3">H12/G12-1</f>
+        <v>4.1010765003353322E-2</v>
+      </c>
+      <c r="I14" s="43">
+        <f t="shared" si="3"/>
+        <v>0.10024053747995643</v>
+      </c>
+      <c r="J14" s="43">
+        <f t="shared" si="3"/>
+        <v>4.7617961866998515E-2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>